<commit_message>
porzingis 2015 class update
</commit_message>
<xml_diff>
--- a/validation.xlsx
+++ b/validation.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\uttam\Desktop\Sports\basketball\bart\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EFD2DFB5-5349-4120-9BE3-9A3CC2C17366}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBAAFDCD-2806-4378-BE67-34F89C9E64C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{8CF2FCA8-9615-4DD6-B0F6-7A2F5E6CE65C}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8CF2FCA8-9615-4DD6-B0F6-7A2F5E6CE65C}"/>
   </bookViews>
   <sheets>
     <sheet name="summary" sheetId="1" r:id="rId1"/>
@@ -560,9 +560,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9E3D10D-0A18-4888-B8BA-67BCEF22A05F}">
   <dimension ref="A1:M13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -601,7 +601,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -642,7 +642,7 @@
         <v>0.3513</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -668,22 +668,22 @@
         <v>1</v>
       </c>
       <c r="I3" s="1">
-        <v>44.944000000000003</v>
+        <v>45.441200000000002</v>
       </c>
       <c r="J3" s="1">
-        <v>20.285299999999999</v>
+        <v>20.629899999999999</v>
       </c>
       <c r="K3" s="1">
-        <v>8.6497999999999902</v>
+        <v>8.8491999999999909</v>
       </c>
       <c r="L3" s="1">
-        <v>3.5250999999999899</v>
+        <v>3.6377999999999999</v>
       </c>
       <c r="M3" s="1">
-        <v>0.32469999999999999</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+        <v>0.34510000000000002</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -724,7 +724,7 @@
         <v>0.29649999999999999</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -765,7 +765,7 @@
         <v>0.28149999999999997</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -806,7 +806,7 @@
         <v>0.3322</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -847,7 +847,7 @@
         <v>0.3982</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -888,7 +888,7 @@
         <v>0.2485</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -929,7 +929,7 @@
         <v>0.1925</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -970,7 +970,7 @@
         <v>0.26439999999999902</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -1011,7 +1011,7 @@
         <v>0.24249999999999999</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>11</v>
       </c>
@@ -1052,7 +1052,7 @@
         <v>0.235599999999999</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>12</v>
       </c>
@@ -1101,9 +1101,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD7FA1E2-9557-425C-9EE9-5E8EDDD2FE6A}">
   <dimension ref="A1:E13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -1118,7 +1118,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -1135,7 +1135,7 @@
         <v>0.71381395210041099</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -1146,13 +1146,13 @@
         <v>5014</v>
       </c>
       <c r="D3" s="1">
-        <v>0.59100532593080202</v>
+        <v>0.59369842964575503</v>
       </c>
       <c r="E3" s="1">
-        <v>0.67103230751124798</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+        <v>0.66999176791022996</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -1169,7 +1169,7 @@
         <v>0.71898230001768104</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -1186,7 +1186,7 @@
         <v>0.70039937526636398</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -1203,7 +1203,7 @@
         <v>0.71364316579987896</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -1220,7 +1220,7 @@
         <v>0.74312921769596296</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -1237,7 +1237,7 @@
         <v>0.73630383429213997</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -1254,7 +1254,7 @@
         <v>0.71637106079276403</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -1271,7 +1271,7 @@
         <v>0.71467497618206499</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -1288,7 +1288,7 @@
         <v>0.70373742526880501</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>11</v>
       </c>
@@ -1305,7 +1305,7 @@
         <v>0.73203595611333605</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>12</v>
       </c>
@@ -1330,9 +1330,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{834031E8-EFDD-445C-BEA4-4000BC5A8F34}">
   <dimension ref="A1:H13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -1356,7 +1356,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -1382,7 +1382,7 @@
         <v>0.205556612948259</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -1393,7 +1393,7 @@
         <v>53</v>
       </c>
       <c r="D3" s="1">
-        <v>0.42304513484516199</v>
+        <v>0.436188441236044</v>
       </c>
       <c r="E3" s="1">
         <v>0.86231649850257597</v>
@@ -1408,7 +1408,7 @@
         <v>0.40032038451271701</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -1434,7 +1434,7 @@
         <v>0.28466497871377799</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -1460,7 +1460,7 @@
         <v>0.370986067151996</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -1486,7 +1486,7 @@
         <v>0.31782730968713402</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -1510,7 +1510,7 @@
       </c>
       <c r="H7" s="1"/>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -1536,7 +1536,7 @@
         <v>0.33729250475845701</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -1562,7 +1562,7 @@
         <v>0.306044563332868</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -1588,7 +1588,7 @@
         <v>0.27551938438899098</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -1614,7 +1614,7 @@
         <v>0.19245008972987501</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>11</v>
       </c>
@@ -1638,7 +1638,7 @@
       </c>
       <c r="H12" s="1"/>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>12</v>
       </c>
@@ -1673,9 +1673,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C0481036-F6AB-449C-BC56-993E67FE8301}">
   <dimension ref="A1:H13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -1699,7 +1699,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -1725,7 +1725,7 @@
         <v>0.169030850945703</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -1736,7 +1736,7 @@
         <v>53</v>
       </c>
       <c r="D3" s="1">
-        <v>0.28094375716441999</v>
+        <v>0.29255900293866</v>
       </c>
       <c r="E3" s="1">
         <v>0.71068968321943604</v>
@@ -1751,7 +1751,7 @@
         <v>0.32992940266093701</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -1777,7 +1777,7 @@
         <v>0.23403649916646899</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -1803,7 +1803,7 @@
         <v>0.30472814416366301</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -1829,7 +1829,7 @@
         <v>0.26100930058746902</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -1853,7 +1853,7 @@
       </c>
       <c r="H7" s="1"/>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -1879,7 +1879,7 @@
         <v>0.27720408594239299</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -1905,7 +1905,7 @@
         <v>0.25122421158813202</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -1931,7 +1931,7 @@
         <v>0.22641670642586301</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -1957,7 +1957,7 @@
         <v>0.158113883008418</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>11</v>
       </c>
@@ -1981,7 +1981,7 @@
       </c>
       <c r="H12" s="1"/>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>12</v>
       </c>
@@ -2013,9 +2013,9 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3208696C-FD95-4C0F-8D26-9B4D6AE84141}">
   <dimension ref="A1:G13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -2036,7 +2036,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -2059,7 +2059,7 @@
         <v>3.9246256248729898E-4</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -2070,19 +2070,19 @@
         <v>5014</v>
       </c>
       <c r="D3" s="1">
-        <v>8.8459283326685206E-3</v>
+        <v>8.78056051455923E-3</v>
       </c>
       <c r="E3" s="1">
-        <v>4.2714272895891499E-3</v>
+        <v>4.1848717969684797E-3</v>
       </c>
       <c r="F3" s="1">
-        <v>1.7300236617471001E-3</v>
+        <v>1.66575752692461E-3</v>
       </c>
       <c r="G3" s="1">
-        <v>5.5645282608695603E-4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+        <v>5.6077966094934199E-4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -2105,7 +2105,7 @@
         <v>8.4019271277697202E-4</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -2128,7 +2128,7 @@
         <v>1.11152014355034E-3</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -2151,7 +2151,7 @@
         <v>5.29679670240744E-4</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -2174,7 +2174,7 @@
         <v>3.0841810576327197E-4</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -2197,7 +2197,7 @@
         <v>5.7541684860967996E-4</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -2220,7 +2220,7 @@
         <v>4.7964939972714799E-4</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -2243,7 +2243,7 @@
         <v>3.27676166894131E-4</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -2266,7 +2266,7 @@
         <v>1.28151464832396E-4</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>11</v>
       </c>
@@ -2289,7 +2289,7 @@
         <v>3.3648135493947598E-5</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>12</v>
       </c>
@@ -2320,9 +2320,9 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26959CBB-4390-4525-A282-958F0D73204D}">
   <dimension ref="A1:G13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -2343,7 +2343,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -2366,7 +2366,7 @@
         <v>1.8359155628506899E-3</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -2377,19 +2377,19 @@
         <v>5014</v>
       </c>
       <c r="D3" s="1">
-        <v>5.5541972140753397E-2</v>
+        <v>5.5386656054931503E-2</v>
       </c>
       <c r="E3" s="1">
-        <v>2.3951399850506299E-2</v>
+        <v>2.3750341739311599E-2</v>
       </c>
       <c r="F3" s="1">
-        <v>1.2946247566846199E-2</v>
+        <v>1.27167538023139E-2</v>
       </c>
       <c r="G3" s="1">
-        <v>2.2842111931303398E-3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+        <v>2.3091143856933901E-3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -2412,7 +2412,7 @@
         <v>4.6051012535165397E-3</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -2435,7 +2435,7 @@
         <v>4.5129289845963899E-3</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -2458,7 +2458,7 @@
         <v>2.41777490178366E-3</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -2481,7 +2481,7 @@
         <v>2.3975376012372899E-3</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -2504,7 +2504,7 @@
         <v>2.45734332225531E-3</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -2527,7 +2527,7 @@
         <v>1.7198690047920801E-3</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -2550,7 +2550,7 @@
         <v>1.45964132611186E-3</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -2573,7 +2573,7 @@
         <v>8.5615411174013605E-4</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>11</v>
       </c>
@@ -2596,7 +2596,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>12</v>
       </c>
@@ -2627,9 +2627,9 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{88E95CE6-CD40-4D98-91F1-85007EDA77BB}">
   <dimension ref="A1:G13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -2650,7 +2650,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -2673,7 +2673,7 @@
         <v>0.99766212644846497</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -2684,19 +2684,19 @@
         <v>5014</v>
       </c>
       <c r="D3" s="1">
-        <v>0.94931321646864697</v>
+        <v>0.94933445172341702</v>
       </c>
       <c r="E3" s="1">
-        <v>0.95980738387514597</v>
+        <v>0.95990762445253197</v>
       </c>
       <c r="F3" s="1">
-        <v>0.93361083361083297</v>
+        <v>0.93392163392163297</v>
       </c>
       <c r="G3" s="1">
-        <v>0.997405707443624</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+        <v>0.99733918712166503</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -2719,7 +2719,7 @@
         <v>0.980984455958549</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -2742,7 +2742,7 @@
         <v>0.99441632928474999</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -2765,7 +2765,7 @@
         <v>0.994871794871794</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -2788,7 +2788,7 @@
         <v>0.959710743801652</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -2811,7 +2811,7 @@
         <v>0.997045891728496</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -2834,7 +2834,7 @@
         <v>0.99980499219968799</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -2857,7 +2857,7 @@
         <v>0.99912229373902794</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -2880,7 +2880,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>11</v>
       </c>
@@ -2901,7 +2901,7 @@
       </c>
       <c r="G12" s="1"/>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>12</v>
       </c>
@@ -2930,9 +2930,9 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E7C1D4F9-388A-41D2-B1F5-AEE3CC4FABF1}">
   <dimension ref="A1:G13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -2953,7 +2953,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -2976,7 +2976,7 @@
         <v>0.170454545454545</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -2987,19 +2987,19 @@
         <v>5014</v>
       </c>
       <c r="D3" s="1">
-        <v>0.36366137538405002</v>
+        <v>0.37069888970507697</v>
       </c>
       <c r="E3" s="1">
-        <v>0.31524000389276602</v>
+        <v>0.33366596199263698</v>
       </c>
       <c r="F3" s="1">
-        <v>0.14177610852731301</v>
+        <v>0.16626336590930799</v>
       </c>
       <c r="G3" s="1">
-        <v>0.16499999999999901</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+        <v>0.16254901960784299</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -3022,7 +3022,7 @@
         <v>6.4644470640920895E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -3045,7 +3045,7 @@
         <v>0.19704202131738299</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -3068,7 +3068,7 @@
         <v>0.26388888888888801</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -3091,7 +3091,7 @@
         <v>5.0761421319796898E-3</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -3114,7 +3114,7 @@
         <v>0.165865384615384</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -3137,7 +3137,7 @@
         <v>0.63888888888888795</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -3160,7 +3160,7 @@
         <v>0.59090909090909005</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -3183,7 +3183,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>11</v>
       </c>
@@ -3206,7 +3206,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>12</v>
       </c>
@@ -3237,9 +3237,9 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82367681-20B8-422B-BAF8-1E957EF58DE1}">
   <dimension ref="A1:G13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -3260,7 +3260,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -3283,7 +3283,7 @@
         <v>0.49600149681275901</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -3294,19 +3294,19 @@
         <v>5014</v>
       </c>
       <c r="D3" s="1">
-        <v>0.81818185977726199</v>
+        <v>0.81841518232205401</v>
       </c>
       <c r="E3" s="1">
-        <v>0.56447017764968199</v>
+        <v>0.56453423261997204</v>
       </c>
       <c r="F3" s="1">
-        <v>0.50325644677389203</v>
+        <v>0.50331052756414696</v>
       </c>
       <c r="G3" s="1">
-        <v>0.49630566224661699</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+        <v>0.49600605193270503</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -3329,7 +3329,7 @@
         <v>0.49280763772352798</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -3352,7 +3352,7 @@
         <v>0.50050768732778494</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -3375,7 +3375,7 @@
         <v>0.50019235883871804</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -3398,7 +3398,7 @@
         <v>0.15971069115011899</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -3421,7 +3421,7 @@
         <v>0.49742029097373303</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -3444,7 +3444,7 @@
         <v>0.50019482709466201</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -3467,7 +3467,7 @@
         <v>0.49830956417099198</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -3490,7 +3490,7 @@
         <v>0.16637591166462501</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>11</v>
       </c>
@@ -3513,7 +3513,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>12</v>
       </c>

</xml_diff>

<commit_message>
conditional p_nba based update
</commit_message>
<xml_diff>
--- a/validation.xlsx
+++ b/validation.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\uttam\Desktop\Sports\basketball\bart\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBAAFDCD-2806-4378-BE67-34F89C9E64C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16D906C1-0C7A-4D9D-AB5D-8F21D8A5FDD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8CF2FCA8-9615-4DD6-B0F6-7A2F5E6CE65C}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="8" xr2:uid="{8CF2FCA8-9615-4DD6-B0F6-7A2F5E6CE65C}"/>
   </bookViews>
   <sheets>
     <sheet name="summary" sheetId="1" r:id="rId1"/>
@@ -197,12 +197,18 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -217,12 +223,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="11" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -609,10 +618,10 @@
         <v>2014</v>
       </c>
       <c r="C2" s="1">
-        <v>4921</v>
+        <v>4751</v>
       </c>
       <c r="D2" s="1">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E2" s="1">
         <v>32</v>
@@ -627,19 +636,19 @@
         <v>2</v>
       </c>
       <c r="I2" s="1">
-        <v>55.8508</v>
+        <v>53.4438999999999</v>
       </c>
       <c r="J2" s="1">
-        <v>25.445899999999899</v>
+        <v>26.486799999999999</v>
       </c>
       <c r="K2" s="1">
-        <v>10.864699999999999</v>
+        <v>11.5878</v>
       </c>
       <c r="L2" s="1">
-        <v>4.4044999999999996</v>
+        <v>4.6981000000000002</v>
       </c>
       <c r="M2" s="1">
-        <v>0.3513</v>
+        <v>0.39400000000000002</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.3">
@@ -650,10 +659,10 @@
         <v>2015</v>
       </c>
       <c r="C3" s="1">
-        <v>5014</v>
+        <v>4848</v>
       </c>
       <c r="D3" s="1">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E3" s="1">
         <v>26</v>
@@ -668,19 +677,19 @@
         <v>1</v>
       </c>
       <c r="I3" s="1">
-        <v>45.441200000000002</v>
+        <v>48.003999999999998</v>
       </c>
       <c r="J3" s="1">
-        <v>20.629899999999999</v>
+        <v>23.073999999999899</v>
       </c>
       <c r="K3" s="1">
-        <v>8.8491999999999909</v>
+        <v>9.8202999999999996</v>
       </c>
       <c r="L3" s="1">
-        <v>3.6377999999999999</v>
+        <v>3.8391000000000002</v>
       </c>
       <c r="M3" s="1">
-        <v>0.34510000000000002</v>
+        <v>0.29430000000000001</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.3">
@@ -691,13 +700,13 @@
         <v>2016</v>
       </c>
       <c r="C4" s="1">
-        <v>4829</v>
+        <v>4709</v>
       </c>
       <c r="D4" s="1">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="E4" s="1">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F4" s="1">
         <v>11</v>
@@ -709,19 +718,19 @@
         <v>0</v>
       </c>
       <c r="I4" s="1">
-        <v>48.482900000000001</v>
+        <v>52.4621</v>
       </c>
       <c r="J4" s="1">
-        <v>21.515999999999998</v>
+        <v>25.564799999999899</v>
       </c>
       <c r="K4" s="1">
-        <v>9.0712999999999901</v>
+        <v>11.2044</v>
       </c>
       <c r="L4" s="1">
-        <v>3.6162999999999998</v>
+        <v>4.5259999999999998</v>
       </c>
       <c r="M4" s="1">
-        <v>0.29649999999999999</v>
+        <v>0.35669999999999902</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.3">
@@ -732,10 +741,10 @@
         <v>2017</v>
       </c>
       <c r="C5" s="1">
-        <v>4946</v>
+        <v>4796</v>
       </c>
       <c r="D5" s="1">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E5" s="1">
         <v>29</v>
@@ -750,19 +759,19 @@
         <v>1</v>
       </c>
       <c r="I5" s="1">
-        <v>51.6282</v>
+        <v>57.664299999999997</v>
       </c>
       <c r="J5" s="1">
-        <v>22.8245</v>
+        <v>27.849599999999999</v>
       </c>
       <c r="K5" s="1">
-        <v>9.3249999999999993</v>
+        <v>11.871700000000001</v>
       </c>
       <c r="L5" s="1">
-        <v>3.6371000000000002</v>
+        <v>4.6639999999999997</v>
       </c>
       <c r="M5" s="1">
-        <v>0.28149999999999997</v>
+        <v>0.33929999999999999</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.3">
@@ -773,7 +782,7 @@
         <v>2018</v>
       </c>
       <c r="C6" s="1">
-        <v>4943</v>
+        <v>4782</v>
       </c>
       <c r="D6" s="1">
         <v>60</v>
@@ -791,19 +800,19 @@
         <v>1</v>
       </c>
       <c r="I6" s="1">
-        <v>57.3004999999999</v>
+        <v>65.572899999999905</v>
       </c>
       <c r="J6" s="1">
-        <v>26.193300000000001</v>
+        <v>32.790999999999997</v>
       </c>
       <c r="K6" s="1">
-        <v>10.875299999999999</v>
+        <v>14.4825</v>
       </c>
       <c r="L6" s="1">
-        <v>4.2797000000000001</v>
+        <v>5.8554000000000004</v>
       </c>
       <c r="M6" s="1">
-        <v>0.3322</v>
+        <v>0.464699999999999</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.3">
@@ -814,7 +823,7 @@
         <v>2019</v>
       </c>
       <c r="C7" s="1">
-        <v>4841</v>
+        <v>4699</v>
       </c>
       <c r="D7" s="1">
         <v>62</v>
@@ -832,19 +841,19 @@
         <v>0</v>
       </c>
       <c r="I7" s="1">
-        <v>65.423599999999894</v>
+        <v>72.174799999999905</v>
       </c>
       <c r="J7" s="1">
-        <v>30.019500000000001</v>
+        <v>35.671199999999999</v>
       </c>
       <c r="K7" s="1">
-        <v>12.545199999999999</v>
+        <v>15.422799999999899</v>
       </c>
       <c r="L7" s="1">
-        <v>4.9380999999999897</v>
+        <v>6.0345000000000004</v>
       </c>
       <c r="M7" s="1">
-        <v>0.3982</v>
+        <v>0.46450000000000002</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.3">
@@ -855,7 +864,7 @@
         <v>2020</v>
       </c>
       <c r="C8" s="1">
-        <v>4855</v>
+        <v>4724</v>
       </c>
       <c r="D8" s="1">
         <v>56</v>
@@ -873,19 +882,19 @@
         <v>0</v>
       </c>
       <c r="I8" s="1">
-        <v>58.0870999999999</v>
+        <v>64.066499999999905</v>
       </c>
       <c r="J8" s="1">
-        <v>24.167999999999999</v>
+        <v>29.863899999999902</v>
       </c>
       <c r="K8" s="1">
-        <v>9.3472000000000008</v>
+        <v>12.0152999999999</v>
       </c>
       <c r="L8" s="1">
-        <v>3.4508000000000001</v>
+        <v>4.4763999999999902</v>
       </c>
       <c r="M8" s="1">
-        <v>0.2485</v>
+        <v>0.30909999999999899</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.3">
@@ -896,7 +905,7 @@
         <v>2021</v>
       </c>
       <c r="C9" s="1">
-        <v>5131</v>
+        <v>4988</v>
       </c>
       <c r="D9" s="1">
         <v>60</v>
@@ -914,19 +923,19 @@
         <v>0</v>
       </c>
       <c r="I9" s="1">
-        <v>50.451900000000002</v>
+        <v>60.684599999999897</v>
       </c>
       <c r="J9" s="1">
-        <v>20.535</v>
+        <v>28.3002</v>
       </c>
       <c r="K9" s="1">
-        <v>7.8236999999999997</v>
+        <v>11.5968</v>
       </c>
       <c r="L9" s="1">
-        <v>2.8458999999999999</v>
+        <v>4.4429999999999996</v>
       </c>
       <c r="M9" s="1">
-        <v>0.1925</v>
+        <v>0.30399999999999999</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.3">
@@ -937,7 +946,7 @@
         <v>2022</v>
       </c>
       <c r="C10" s="1">
-        <v>5129</v>
+        <v>5025</v>
       </c>
       <c r="D10" s="1">
         <v>42</v>
@@ -955,19 +964,19 @@
         <v>0</v>
       </c>
       <c r="I10" s="1">
-        <v>54.310499999999998</v>
+        <v>64.298199999999994</v>
       </c>
       <c r="J10" s="1">
-        <v>23.465199999999999</v>
+        <v>30.8325</v>
       </c>
       <c r="K10" s="1">
-        <v>9.3996999999999993</v>
+        <v>12.632300000000001</v>
       </c>
       <c r="L10" s="1">
-        <v>3.5752000000000002</v>
+        <v>4.8186</v>
       </c>
       <c r="M10" s="1">
-        <v>0.26439999999999902</v>
+        <v>0.32329999999999998</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.3">
@@ -978,7 +987,7 @@
         <v>2023</v>
       </c>
       <c r="C11" s="1">
-        <v>5161</v>
+        <v>5039</v>
       </c>
       <c r="D11" s="1">
         <v>37</v>
@@ -996,19 +1005,19 @@
         <v>1</v>
       </c>
       <c r="I11" s="1">
-        <v>52.577799999999897</v>
+        <v>62.064499999999903</v>
       </c>
       <c r="J11" s="1">
-        <v>23.200700000000001</v>
+        <v>29.16</v>
       </c>
       <c r="K11" s="1">
-        <v>9.2614000000000001</v>
+        <v>12.165699999999999</v>
       </c>
       <c r="L11" s="1">
-        <v>3.5086999999999899</v>
+        <v>4.6256999999999904</v>
       </c>
       <c r="M11" s="1">
-        <v>0.24249999999999999</v>
+        <v>0.31069999999999998</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.3">
@@ -1019,7 +1028,7 @@
         <v>2024</v>
       </c>
       <c r="C12" s="1">
-        <v>5122</v>
+        <v>5011</v>
       </c>
       <c r="D12" s="1">
         <v>28</v>
@@ -1037,19 +1046,19 @@
         <v>0</v>
       </c>
       <c r="I12" s="1">
-        <v>50.265899999999903</v>
+        <v>62.259699999999903</v>
       </c>
       <c r="J12" s="1">
-        <v>20.382199999999902</v>
+        <v>27.849999999999898</v>
       </c>
       <c r="K12" s="1">
-        <v>7.8174000000000001</v>
+        <v>10.956200000000001</v>
       </c>
       <c r="L12" s="1">
-        <v>2.9885000000000002</v>
+        <v>3.9201999999999901</v>
       </c>
       <c r="M12" s="1">
-        <v>0.235599999999999</v>
+        <v>0.2487</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.3">
@@ -1060,7 +1069,7 @@
         <v>2025</v>
       </c>
       <c r="C13" s="1">
-        <v>5114</v>
+        <v>5001</v>
       </c>
       <c r="D13" s="1">
         <v>26</v>
@@ -1078,19 +1087,19 @@
         <v>0</v>
       </c>
       <c r="I13" s="1">
-        <v>57.218299999999999</v>
+        <v>69.762699999999995</v>
       </c>
       <c r="J13" s="1">
-        <v>25.117999999999999</v>
+        <v>32.362699999999997</v>
       </c>
       <c r="K13" s="1">
-        <v>10.159000000000001</v>
+        <v>13.1282</v>
       </c>
       <c r="L13" s="1">
-        <v>3.9390999999999998</v>
+        <v>4.9113999999999898</v>
       </c>
       <c r="M13" s="1">
-        <v>0.30590000000000001</v>
+        <v>0.32539999999999902</v>
       </c>
     </row>
   </sheetData>
@@ -1126,13 +1135,13 @@
         <v>2014</v>
       </c>
       <c r="C2" s="1">
-        <v>4921</v>
+        <v>4751</v>
       </c>
       <c r="D2" s="1">
-        <v>0.57262845471944901</v>
+        <v>0.62904738429135298</v>
       </c>
       <c r="E2" s="1">
-        <v>0.71381395210041099</v>
+        <v>0.57606815192166105</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
@@ -1143,13 +1152,13 @@
         <v>2015</v>
       </c>
       <c r="C3" s="1">
-        <v>5014</v>
+        <v>4848</v>
       </c>
       <c r="D3" s="1">
-        <v>0.59369842964575503</v>
+        <v>0.66085125806261003</v>
       </c>
       <c r="E3" s="1">
-        <v>0.66999176791022996</v>
+        <v>0.55285540444495895</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
@@ -1160,13 +1169,13 @@
         <v>2016</v>
       </c>
       <c r="C4" s="1">
-        <v>4829</v>
+        <v>4709</v>
       </c>
       <c r="D4" s="1">
-        <v>0.55901500762131795</v>
+        <v>0.60289537688969297</v>
       </c>
       <c r="E4" s="1">
-        <v>0.71898230001768104</v>
+        <v>0.60922744434750498</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
@@ -1177,13 +1186,13 @@
         <v>2017</v>
       </c>
       <c r="C5" s="1">
-        <v>4946</v>
+        <v>4796</v>
       </c>
       <c r="D5" s="1">
-        <v>0.59009683099139798</v>
+        <v>0.62910354539779401</v>
       </c>
       <c r="E5" s="1">
-        <v>0.70039937526636398</v>
+        <v>0.60123767427657604</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
@@ -1194,13 +1203,13 @@
         <v>2018</v>
       </c>
       <c r="C6" s="1">
-        <v>4943</v>
+        <v>4782</v>
       </c>
       <c r="D6" s="1">
-        <v>0.60333573314661304</v>
+        <v>0.64931154434332605</v>
       </c>
       <c r="E6" s="1">
-        <v>0.71364316579987896</v>
+        <v>0.59109916966222098</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
@@ -1211,13 +1220,13 @@
         <v>2019</v>
       </c>
       <c r="C7" s="1">
-        <v>4841</v>
+        <v>4699</v>
       </c>
       <c r="D7" s="1">
-        <v>0.59072167143405896</v>
+        <v>0.61803203724831901</v>
       </c>
       <c r="E7" s="1">
-        <v>0.74312921769596296</v>
+        <v>0.59789898280258202</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
@@ -1228,13 +1237,13 @@
         <v>2020</v>
       </c>
       <c r="C8" s="1">
-        <v>4855</v>
+        <v>4724</v>
       </c>
       <c r="D8" s="1">
-        <v>0.59025162286133803</v>
+        <v>0.62947983001024399</v>
       </c>
       <c r="E8" s="1">
-        <v>0.73630383429213997</v>
+        <v>0.60319535411104697</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
@@ -1245,13 +1254,13 @@
         <v>2021</v>
       </c>
       <c r="C9" s="1">
-        <v>5131</v>
+        <v>4988</v>
       </c>
       <c r="D9" s="1">
-        <v>0.59114689972465295</v>
+        <v>0.64514347711221798</v>
       </c>
       <c r="E9" s="1">
-        <v>0.71637106079276403</v>
+        <v>0.59707705975019898</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
@@ -1262,13 +1271,13 @@
         <v>2022</v>
       </c>
       <c r="C10" s="1">
-        <v>5129</v>
+        <v>5025</v>
       </c>
       <c r="D10" s="1">
-        <v>0.56491579691364402</v>
+        <v>0.60558041644641203</v>
       </c>
       <c r="E10" s="1">
-        <v>0.71467497618206499</v>
+        <v>0.56057537235124399</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
@@ -1279,13 +1288,13 @@
         <v>2023</v>
       </c>
       <c r="C11" s="1">
-        <v>5161</v>
+        <v>5039</v>
       </c>
       <c r="D11" s="1">
-        <v>0.55897849677761102</v>
+        <v>0.629025124724096</v>
       </c>
       <c r="E11" s="1">
-        <v>0.70373742526880501</v>
+        <v>0.51488837423241396</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
@@ -1296,13 +1305,13 @@
         <v>2024</v>
       </c>
       <c r="C12" s="1">
-        <v>5122</v>
+        <v>5011</v>
       </c>
       <c r="D12" s="1">
-        <v>0.48084919936346898</v>
+        <v>0.541899488078597</v>
       </c>
       <c r="E12" s="1">
-        <v>0.73203595611333605</v>
+        <v>0.48946260685493798</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
@@ -1313,13 +1322,13 @@
         <v>2025</v>
       </c>
       <c r="C13" s="1">
-        <v>5114</v>
+        <v>5001</v>
       </c>
       <c r="D13" s="1">
-        <v>0.46710625006842399</v>
+        <v>0.55559465781943596</v>
       </c>
       <c r="E13" s="1">
-        <v>0.74837017265326999</v>
+        <v>0.45090418187128001</v>
       </c>
     </row>
   </sheetData>
@@ -1364,22 +1373,22 @@
         <v>2014</v>
       </c>
       <c r="C2" s="1">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="D2" s="1">
-        <v>0.64432877013657797</v>
+        <v>0.62594414708144097</v>
       </c>
       <c r="E2" s="1">
-        <v>0.78254065159730002</v>
+        <v>0.78078528959579996</v>
       </c>
       <c r="F2" s="1">
-        <v>0.710777844271274</v>
+        <v>0.72207366267684203</v>
       </c>
       <c r="G2" s="1">
-        <v>0.48492270581866198</v>
+        <v>0.49462349966121899</v>
       </c>
       <c r="H2" s="1">
-        <v>0.205556612948259</v>
+        <v>0.21004201260420099</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -1390,22 +1399,22 @@
         <v>2015</v>
       </c>
       <c r="C3" s="1">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D3" s="1">
-        <v>0.436188441236044</v>
+        <v>0.477407969966472</v>
       </c>
       <c r="E3" s="1">
-        <v>0.86231649850257597</v>
+        <v>0.86469203054747001</v>
       </c>
       <c r="F3" s="1">
-        <v>0.74535599249993001</v>
+        <v>0.75498344352707403</v>
       </c>
       <c r="G3" s="1">
-        <v>0.54889165714378496</v>
+        <v>0.55815630565143803</v>
       </c>
       <c r="H3" s="1">
-        <v>0.40032038451271701</v>
+        <v>0.407619732292054</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
@@ -1416,22 +1425,22 @@
         <v>2016</v>
       </c>
       <c r="C4" s="1">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="D4" s="1">
-        <v>0.33701812972932499</v>
+        <v>0.34940771025721501</v>
       </c>
       <c r="E4" s="1">
-        <v>0.79793288796170803</v>
+        <v>0.804153333762198</v>
       </c>
       <c r="F4" s="1">
-        <v>0.72015176225511202</v>
+        <v>0.72738405872799405</v>
       </c>
       <c r="G4" s="1">
-        <v>0.544383562614839</v>
+        <v>0.55112199757907798</v>
       </c>
       <c r="H4" s="1">
-        <v>0.28466497871377799</v>
+        <v>0.28858673308160998</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
@@ -1442,22 +1451,22 @@
         <v>2017</v>
       </c>
       <c r="C5" s="1">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="D5" s="1">
-        <v>0.573899445525338</v>
+        <v>0.54723873799559097</v>
       </c>
       <c r="E5" s="1">
-        <v>0.76452257881580099</v>
+        <v>0.75909124102120995</v>
       </c>
       <c r="F5" s="1">
-        <v>0.64863834863279002</v>
+        <v>0.65495298658311796</v>
       </c>
       <c r="G5" s="1">
-        <v>0.48135986234123201</v>
+        <v>0.48671371862979002</v>
       </c>
       <c r="H5" s="1">
-        <v>0.370986067151996</v>
+        <v>0.37530475421527099</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
@@ -1471,7 +1480,7 @@
         <v>86</v>
       </c>
       <c r="D6" s="1">
-        <v>0.57336541246929096</v>
+        <v>0.55108712622965195</v>
       </c>
       <c r="E6" s="1">
         <v>0.77694987973398899</v>
@@ -1494,19 +1503,19 @@
         <v>2019</v>
       </c>
       <c r="C7" s="1">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="D7" s="1">
-        <v>0.41282836079190599</v>
+        <v>0.39523432861288099</v>
       </c>
       <c r="E7" s="1">
-        <v>0.80638606037969895</v>
+        <v>0.790617088196229</v>
       </c>
       <c r="F7" s="1">
-        <v>0.57004432835591101</v>
-      </c>
-      <c r="G7" s="1">
-        <v>1.79461500985255E-3</v>
+        <v>0.547311688975891</v>
+      </c>
+      <c r="G7" s="3">
+        <v>0</v>
       </c>
       <c r="H7" s="1"/>
     </row>
@@ -1518,22 +1527,22 @@
         <v>2020</v>
       </c>
       <c r="C8" s="1">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D8" s="1">
-        <v>0.36889341552695398</v>
+        <v>0.33266473252900203</v>
       </c>
       <c r="E8" s="1">
-        <v>0.81384130046198899</v>
+        <v>0.81656916808001601</v>
       </c>
       <c r="F8" s="1">
-        <v>0.65226876780553</v>
+        <v>0.65570046591086995</v>
       </c>
       <c r="G8" s="1">
-        <v>0.50090826596203297</v>
+        <v>0.50389662287356596</v>
       </c>
       <c r="H8" s="1">
-        <v>0.33729250475845701</v>
+        <v>0.33944142888212098</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
@@ -1544,22 +1553,22 @@
         <v>2021</v>
       </c>
       <c r="C9" s="1">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D9" s="1">
-        <v>0.52437527773238402</v>
+        <v>0.53746735072179497</v>
       </c>
       <c r="E9" s="1">
-        <v>0.84780829697410398</v>
+        <v>0.85083079603306599</v>
       </c>
       <c r="F9" s="1">
-        <v>0.66947450639184303</v>
+        <v>0.67512747051891997</v>
       </c>
       <c r="G9" s="1">
-        <v>0.42553769653796603</v>
+        <v>0.42986347681054698</v>
       </c>
       <c r="H9" s="1">
-        <v>0.306044563332868</v>
+        <v>0.30927685641354302</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
@@ -1573,7 +1582,7 @@
         <v>77</v>
       </c>
       <c r="D10" s="1">
-        <v>0.33443092717825701</v>
+        <v>0.33563602272541998</v>
       </c>
       <c r="E10" s="1">
         <v>0.79280672936186503</v>
@@ -1596,22 +1605,22 @@
         <v>2023</v>
       </c>
       <c r="C11" s="1">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D11" s="1">
-        <v>0.480519937308237</v>
+        <v>0.45808355922982003</v>
       </c>
       <c r="E11" s="1">
-        <v>0.75005860061734897</v>
+        <v>0.75319830875254301</v>
       </c>
       <c r="F11" s="1">
-        <v>0.57286671883027496</v>
+        <v>0.57596073584122798</v>
       </c>
       <c r="G11" s="1">
-        <v>0.32908687544372001</v>
+        <v>0.331082141794728</v>
       </c>
       <c r="H11" s="1">
-        <v>0.19245008972987501</v>
+        <v>0.19364916731036999</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
@@ -1625,7 +1634,7 @@
         <v>81</v>
       </c>
       <c r="D12" s="1">
-        <v>0.50199869025200605</v>
+        <v>0.498890490482501</v>
       </c>
       <c r="E12" s="1">
         <v>0.78106400224933903</v>
@@ -1646,19 +1655,19 @@
         <v>2025</v>
       </c>
       <c r="C13" s="1">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D13" s="1">
-        <v>0.60712244176604102</v>
+        <v>0.603368585810375</v>
       </c>
       <c r="E13" s="1">
-        <v>0.79814985395523896</v>
+        <v>0.80077920946439296</v>
       </c>
       <c r="F13" s="1">
-        <v>0.60314788851100298</v>
+        <v>0.60613447995959502</v>
       </c>
       <c r="G13" s="1">
-        <v>0.31962394847466902</v>
+        <v>0.32145135081780801</v>
       </c>
       <c r="H13" s="1"/>
     </row>
@@ -1707,22 +1716,22 @@
         <v>2014</v>
       </c>
       <c r="C2" s="1">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="D2" s="1">
-        <v>0.46424895393115401</v>
+        <v>0.43452722024858798</v>
       </c>
       <c r="E2" s="1">
-        <v>0.64348945208778596</v>
+        <v>0.64224842494840795</v>
       </c>
       <c r="F2" s="1">
-        <v>0.58447832024147595</v>
+        <v>0.59395416221405295</v>
       </c>
       <c r="G2" s="1">
-        <v>0.39875582902338103</v>
+        <v>0.40686110231961498</v>
       </c>
       <c r="H2" s="1">
-        <v>0.169030850945703</v>
+        <v>0.172773685116272</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -1733,22 +1742,22 @@
         <v>2015</v>
       </c>
       <c r="C3" s="1">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D3" s="1">
-        <v>0.29255900293866</v>
+        <v>0.326659040885871</v>
       </c>
       <c r="E3" s="1">
-        <v>0.71068968321943604</v>
+        <v>0.71290623094320504</v>
       </c>
       <c r="F3" s="1">
-        <v>0.61429511683395099</v>
+        <v>0.62245560515763398</v>
       </c>
       <c r="G3" s="1">
-        <v>0.45237640543200502</v>
+        <v>0.46017899330842199</v>
       </c>
       <c r="H3" s="1">
-        <v>0.32992940266093701</v>
+        <v>0.33606722016672202</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
@@ -1759,22 +1768,22 @@
         <v>2016</v>
       </c>
       <c r="C4" s="1">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="D4" s="1">
-        <v>0.244858212561824</v>
+        <v>0.24263824351084101</v>
       </c>
       <c r="E4" s="1">
-        <v>0.65601824471746994</v>
+        <v>0.66126173391883303</v>
       </c>
       <c r="F4" s="1">
-        <v>0.59207071438251402</v>
+        <v>0.59813374353507198</v>
       </c>
       <c r="G4" s="1">
-        <v>0.44756339109156701</v>
+        <v>0.45319203741275799</v>
       </c>
       <c r="H4" s="1">
-        <v>0.23403649916646899</v>
+        <v>0.237307184452895</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
@@ -1785,22 +1794,22 @@
         <v>2017</v>
       </c>
       <c r="C5" s="1">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="D5" s="1">
-        <v>0.40582278280961198</v>
+        <v>0.37861263631915598</v>
       </c>
       <c r="E5" s="1">
-        <v>0.62797923491370999</v>
+        <v>0.62360956446232296</v>
       </c>
       <c r="F5" s="1">
-        <v>0.53279186932718603</v>
+        <v>0.53805777834681101</v>
       </c>
       <c r="G5" s="1">
-        <v>0.39538923564485901</v>
+        <v>0.39984564923214599</v>
       </c>
       <c r="H5" s="1">
-        <v>0.30472814416366301</v>
+        <v>0.308320820566924</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
@@ -1814,7 +1823,7 @@
         <v>86</v>
       </c>
       <c r="D6" s="1">
-        <v>0.40597209313837601</v>
+        <v>0.38515301143897201</v>
       </c>
       <c r="E6" s="1">
         <v>0.63805449852787199</v>
@@ -1837,19 +1846,19 @@
         <v>2019</v>
       </c>
       <c r="C7" s="1">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="D7" s="1">
-        <v>0.291886610846676</v>
+        <v>0.272717258577789</v>
       </c>
       <c r="E7" s="1">
-        <v>0.66176217730659703</v>
+        <v>0.64896076832351102</v>
       </c>
       <c r="F7" s="1">
-        <v>0.46780790793488902</v>
+        <v>0.44924884560814998</v>
       </c>
       <c r="G7" s="1">
-        <v>1.4727540500736301E-3</v>
+        <v>-9.2538005358879294E-2</v>
       </c>
       <c r="H7" s="1"/>
     </row>
@@ -1861,22 +1870,22 @@
         <v>2020</v>
       </c>
       <c r="C8" s="1">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D8" s="1">
-        <v>0.252413585988912</v>
+        <v>0.226994101530995</v>
       </c>
       <c r="E8" s="1">
-        <v>0.66885605405993798</v>
+        <v>0.67115605521402399</v>
       </c>
       <c r="F8" s="1">
-        <v>0.536067552695209</v>
+        <v>0.53893455117523303</v>
       </c>
       <c r="G8" s="1">
-        <v>0.41167181614791898</v>
+        <v>0.41416365307874498</v>
       </c>
       <c r="H8" s="1">
-        <v>0.27720408594239299</v>
+        <v>0.27899433298516602</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
@@ -1887,22 +1896,22 @@
         <v>2021</v>
       </c>
       <c r="C9" s="1">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D9" s="1">
-        <v>0.38465154889666298</v>
+        <v>0.38567776545570798</v>
       </c>
       <c r="E9" s="1">
-        <v>0.69594430518779904</v>
+        <v>0.69850704213492898</v>
       </c>
       <c r="F9" s="1">
-        <v>0.54955462438231795</v>
+        <v>0.55425978313775104</v>
       </c>
       <c r="G9" s="1">
-        <v>0.34931309071321398</v>
+        <v>0.35290526284276902</v>
       </c>
       <c r="H9" s="1">
-        <v>0.25122421158813202</v>
+        <v>0.25390719656769101</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
@@ -1916,7 +1925,7 @@
         <v>77</v>
       </c>
       <c r="D10" s="1">
-        <v>0.22594428632852101</v>
+        <v>0.238959610610778</v>
       </c>
       <c r="E10" s="1">
         <v>0.65151382684907699</v>
@@ -1939,22 +1948,22 @@
         <v>2023</v>
       </c>
       <c r="C11" s="1">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D11" s="1">
-        <v>0.33122235901430902</v>
+        <v>0.31378928651260302</v>
       </c>
       <c r="E11" s="1">
-        <v>0.61623602251331999</v>
+        <v>0.61886390659923696</v>
       </c>
       <c r="F11" s="1">
-        <v>0.47065803652096699</v>
+        <v>0.47323700397152502</v>
       </c>
       <c r="G11" s="1">
-        <v>0.27037245758912798</v>
+        <v>0.27203298957969901</v>
       </c>
       <c r="H11" s="1">
-        <v>0.158113883008418</v>
+        <v>0.15911145683514599</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
@@ -1968,7 +1977,7 @@
         <v>81</v>
       </c>
       <c r="D12" s="1">
-        <v>0.35392224169409497</v>
+        <v>0.35447036381543701</v>
       </c>
       <c r="E12" s="1">
         <v>0.64166065413248397</v>
@@ -1989,19 +1998,19 @@
         <v>2025</v>
       </c>
       <c r="C13" s="1">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D13" s="1">
-        <v>0.441361955763799</v>
+        <v>0.43917888187085602</v>
       </c>
       <c r="E13" s="1">
-        <v>0.65550886855228696</v>
+        <v>0.65771383810017003</v>
       </c>
       <c r="F13" s="1">
-        <v>0.49535659000411397</v>
+        <v>0.49784388818701297</v>
       </c>
       <c r="G13" s="1">
-        <v>0.26250250098848599</v>
+        <v>0.26402159198198499</v>
       </c>
       <c r="H13" s="1"/>
     </row>
@@ -2044,19 +2053,19 @@
         <v>2014</v>
       </c>
       <c r="C2" s="1">
-        <v>4921</v>
+        <v>4751</v>
       </c>
       <c r="D2" s="1">
-        <v>8.8783498963625196E-3</v>
+        <v>8.7703257566828004E-3</v>
       </c>
       <c r="E2" s="1">
-        <v>5.1238380918512396E-3</v>
+        <v>5.1325873416122898E-3</v>
       </c>
       <c r="F2" s="1">
-        <v>1.59728175370859E-3</v>
+        <v>1.61763531046095E-3</v>
       </c>
       <c r="G2" s="1">
-        <v>3.9246256248729898E-4</v>
+        <v>3.8585455062092102E-4</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
@@ -2067,19 +2076,19 @@
         <v>2015</v>
       </c>
       <c r="C3" s="1">
-        <v>5014</v>
+        <v>4848</v>
       </c>
       <c r="D3" s="1">
-        <v>8.78056051455923E-3</v>
+        <v>8.5543201485148504E-3</v>
       </c>
       <c r="E3" s="1">
-        <v>4.1848717969684797E-3</v>
+        <v>4.2192096947194701E-3</v>
       </c>
       <c r="F3" s="1">
-        <v>1.66575752692461E-3</v>
+        <v>1.54858567450495E-3</v>
       </c>
       <c r="G3" s="1">
-        <v>5.6077966094934199E-4</v>
+        <v>5.4681490717821695E-4</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
@@ -2090,19 +2099,19 @@
         <v>2016</v>
       </c>
       <c r="C4" s="1">
-        <v>4829</v>
+        <v>4709</v>
       </c>
       <c r="D4" s="1">
-        <v>9.8938184530958703E-3</v>
+        <v>9.3976851794436104E-3</v>
       </c>
       <c r="E4" s="1">
-        <v>5.0721005342721E-3</v>
+        <v>4.9817966744531697E-3</v>
       </c>
       <c r="F4" s="1">
-        <v>1.91321255539449E-3</v>
+        <v>1.90757082607772E-3</v>
       </c>
       <c r="G4" s="1">
-        <v>8.4019271277697202E-4</v>
+        <v>8.0957699299214197E-4</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
@@ -2113,19 +2122,19 @@
         <v>2017</v>
       </c>
       <c r="C5" s="1">
-        <v>4946</v>
+        <v>4796</v>
       </c>
       <c r="D5" s="1">
-        <v>9.1312717792155201E-3</v>
+        <v>9.4169567410341895E-3</v>
       </c>
       <c r="E5" s="1">
-        <v>4.8025344177112803E-3</v>
+        <v>5.2780685362802298E-3</v>
       </c>
       <c r="F5" s="1">
-        <v>2.1900323291548702E-3</v>
+        <v>2.3667525750625498E-3</v>
       </c>
       <c r="G5" s="1">
-        <v>1.11152014355034E-3</v>
+        <v>1.1824180442035E-3</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
@@ -2136,19 +2145,19 @@
         <v>2018</v>
       </c>
       <c r="C6" s="1">
-        <v>4943</v>
+        <v>4782</v>
       </c>
       <c r="D6" s="1">
-        <v>1.0121301406028699E-2</v>
+        <v>1.03612465014638E-2</v>
       </c>
       <c r="E6" s="1">
-        <v>3.87079550273113E-3</v>
+        <v>4.2306421790045999E-3</v>
       </c>
       <c r="F6" s="1">
-        <v>1.26603937891968E-3</v>
+        <v>1.3743331932245899E-3</v>
       </c>
       <c r="G6" s="1">
-        <v>5.29679670240744E-4</v>
+        <v>5.5691902551233802E-4</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
@@ -2159,19 +2168,19 @@
         <v>2019</v>
       </c>
       <c r="C7" s="1">
-        <v>4841</v>
+        <v>4699</v>
       </c>
       <c r="D7" s="1">
-        <v>1.0987743536459401E-2</v>
+        <v>1.0995319646733301E-2</v>
       </c>
       <c r="E7" s="1">
-        <v>4.6830852199958601E-3</v>
+        <v>5.1174458565652198E-3</v>
       </c>
       <c r="F7" s="1">
-        <v>1.09941110927494E-3</v>
+        <v>1.09894871674824E-3</v>
       </c>
       <c r="G7" s="1">
-        <v>3.0841810576327197E-4</v>
+        <v>3.1174109172164198E-4</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
@@ -2182,19 +2191,19 @@
         <v>2020</v>
       </c>
       <c r="C8" s="1">
-        <v>4855</v>
+        <v>4724</v>
       </c>
       <c r="D8" s="1">
-        <v>9.6159061853759008E-3</v>
+        <v>9.6337265050804397E-3</v>
       </c>
       <c r="E8" s="1">
-        <v>4.5395590978372802E-3</v>
+        <v>4.6411294602032097E-3</v>
       </c>
       <c r="F8" s="1">
-        <v>1.40399819155509E-3</v>
+        <v>1.44193567950889E-3</v>
       </c>
       <c r="G8" s="1">
-        <v>5.7541684860967996E-4</v>
+        <v>5.8202903471634196E-4</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
@@ -2205,19 +2214,19 @@
         <v>2021</v>
       </c>
       <c r="C9" s="1">
-        <v>5131</v>
+        <v>4988</v>
       </c>
       <c r="D9" s="1">
-        <v>8.7352198928084199E-3</v>
+        <v>8.9840786968724898E-3</v>
       </c>
       <c r="E9" s="1">
-        <v>4.5705718339504901E-3</v>
+        <v>4.6246249759422601E-3</v>
       </c>
       <c r="F9" s="1">
-        <v>1.09998344767101E-3</v>
+        <v>1.21170321972734E-3</v>
       </c>
       <c r="G9" s="1">
-        <v>4.7964939972714799E-4</v>
+        <v>5.4884958700882102E-4</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
@@ -2228,19 +2237,19 @@
         <v>2022</v>
       </c>
       <c r="C10" s="1">
-        <v>5129</v>
+        <v>5025</v>
       </c>
       <c r="D10" s="1">
-        <v>7.3407844121661098E-3</v>
+        <v>7.5338970388059701E-3</v>
       </c>
       <c r="E10" s="1">
-        <v>3.7558332696431998E-3</v>
+        <v>3.9273243482586999E-3</v>
       </c>
       <c r="F10" s="1">
-        <v>1.08081573211152E-3</v>
+        <v>1.14787724378109E-3</v>
       </c>
       <c r="G10" s="1">
-        <v>3.27676166894131E-4</v>
+        <v>3.6001286766169103E-4</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
@@ -2251,19 +2260,19 @@
         <v>2023</v>
       </c>
       <c r="C11" s="1">
-        <v>5161</v>
+        <v>5039</v>
       </c>
       <c r="D11" s="1">
-        <v>6.0152762875411697E-3</v>
+        <v>5.9808137348680299E-3</v>
       </c>
       <c r="E11" s="1">
-        <v>2.52500853904282E-3</v>
+        <v>2.67862721174836E-3</v>
       </c>
       <c r="F11" s="1">
-        <v>5.4414315055221802E-4</v>
+        <v>6.0703774359991997E-4</v>
       </c>
       <c r="G11" s="1">
-        <v>1.28151464832396E-4</v>
+        <v>1.3579637031156899E-4</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
@@ -2274,19 +2283,19 @@
         <v>2024</v>
       </c>
       <c r="C12" s="1">
-        <v>5122</v>
+        <v>5011</v>
       </c>
       <c r="D12" s="1">
-        <v>5.0320439847715698E-3</v>
+        <v>5.43531035521852E-3</v>
       </c>
       <c r="E12" s="1">
-        <v>1.7236147051932799E-3</v>
+        <v>1.9317367910596599E-3</v>
       </c>
       <c r="F12" s="1">
-        <v>5.2869731354939398E-4</v>
+        <v>5.7211953701855902E-4</v>
       </c>
       <c r="G12" s="2">
-        <v>3.3648135493947598E-5</v>
+        <v>3.2801388944322401E-5</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
@@ -2297,19 +2306,19 @@
         <v>2025</v>
       </c>
       <c r="C13" s="1">
-        <v>5114</v>
+        <v>5001</v>
       </c>
       <c r="D13" s="1">
-        <v>3.77344320883848E-3</v>
+        <v>4.16214099380124E-3</v>
       </c>
       <c r="E13" s="1">
-        <v>1.3744470238560801E-3</v>
+        <v>1.6301397540491899E-3</v>
       </c>
       <c r="F13" s="1">
-        <v>4.20913640985529E-4</v>
+        <v>4.8074812237552402E-4</v>
       </c>
       <c r="G13" s="2">
-        <v>7.1236173249902197E-5</v>
+        <v>7.0643047390521894E-5</v>
       </c>
     </row>
   </sheetData>
@@ -2351,19 +2360,19 @@
         <v>2014</v>
       </c>
       <c r="C2" s="1">
-        <v>4921</v>
+        <v>4751</v>
       </c>
       <c r="D2" s="1">
-        <v>4.9715254814285598E-2</v>
+        <v>4.3188447367164998E-2</v>
       </c>
       <c r="E2" s="1">
-        <v>3.33357742591852E-2</v>
+        <v>2.2249314904429999E-2</v>
       </c>
       <c r="F2" s="1">
-        <v>1.30105635285361E-2</v>
+        <v>1.3399843542969799E-2</v>
       </c>
       <c r="G2" s="1">
-        <v>1.8359155628506899E-3</v>
+        <v>1.90267719995262E-3</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
@@ -2374,19 +2383,19 @@
         <v>2015</v>
       </c>
       <c r="C3" s="1">
-        <v>5014</v>
+        <v>4848</v>
       </c>
       <c r="D3" s="1">
-        <v>5.5386656054931503E-2</v>
+        <v>4.7539466755377499E-2</v>
       </c>
       <c r="E3" s="1">
-        <v>2.3750341739311599E-2</v>
+        <v>2.32684068453647E-2</v>
       </c>
       <c r="F3" s="1">
-        <v>1.27167538023139E-2</v>
+        <v>6.1697231374238997E-3</v>
       </c>
       <c r="G3" s="1">
-        <v>2.3091143856933901E-3</v>
+        <v>2.2852064309027598E-3</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
@@ -2397,19 +2406,19 @@
         <v>2016</v>
       </c>
       <c r="C4" s="1">
-        <v>4829</v>
+        <v>4709</v>
       </c>
       <c r="D4" s="1">
-        <v>6.0786695474619998E-2</v>
+        <v>5.8168132894369499E-2</v>
       </c>
       <c r="E4" s="1">
-        <v>4.7380959000200201E-2</v>
+        <v>4.0979722016766897E-2</v>
       </c>
       <c r="F4" s="1">
-        <v>8.76949555018669E-3</v>
+        <v>7.65552404904954E-3</v>
       </c>
       <c r="G4" s="1">
-        <v>4.6051012535165397E-3</v>
+        <v>3.85268638539889E-3</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
@@ -2420,19 +2429,19 @@
         <v>2017</v>
       </c>
       <c r="C5" s="1">
-        <v>4946</v>
+        <v>4796</v>
       </c>
       <c r="D5" s="1">
-        <v>4.8996082457169597E-2</v>
+        <v>4.18516679089092E-2</v>
       </c>
       <c r="E5" s="1">
-        <v>2.7736026322010901E-2</v>
+        <v>2.7141402339237199E-2</v>
       </c>
       <c r="F5" s="1">
-        <v>9.5877420000581807E-3</v>
+        <v>1.0047517026618999E-2</v>
       </c>
       <c r="G5" s="1">
-        <v>4.5129289845963899E-3</v>
+        <v>4.8556008435036799E-3</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
@@ -2443,19 +2452,19 @@
         <v>2018</v>
       </c>
       <c r="C6" s="1">
-        <v>4943</v>
+        <v>4782</v>
       </c>
       <c r="D6" s="1">
-        <v>4.8793954146253399E-2</v>
+        <v>4.7347082960174799E-2</v>
       </c>
       <c r="E6" s="1">
-        <v>2.3665252131973302E-2</v>
+        <v>1.93731275074145E-2</v>
       </c>
       <c r="F6" s="1">
-        <v>6.3068590874193796E-3</v>
+        <v>6.9502204840597697E-3</v>
       </c>
       <c r="G6" s="1">
-        <v>2.41777490178366E-3</v>
+        <v>2.7195977107642298E-3</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
@@ -2466,19 +2475,19 @@
         <v>2019</v>
       </c>
       <c r="C7" s="1">
-        <v>4841</v>
+        <v>4699</v>
       </c>
       <c r="D7" s="1">
-        <v>6.7927460764939607E-2</v>
+        <v>4.7001191339858299E-2</v>
       </c>
       <c r="E7" s="1">
-        <v>2.61303848573009E-2</v>
+        <v>2.7412253369273599E-2</v>
       </c>
       <c r="F7" s="1">
-        <v>5.7855324728471403E-3</v>
+        <v>6.2625678073991798E-3</v>
       </c>
       <c r="G7" s="1">
-        <v>2.3975376012372899E-3</v>
+        <v>2.6975896300700198E-3</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
@@ -2489,19 +2498,19 @@
         <v>2020</v>
       </c>
       <c r="C8" s="1">
-        <v>4855</v>
+        <v>4724</v>
       </c>
       <c r="D8" s="1">
-        <v>4.3146216897040901E-2</v>
+        <v>3.7106502114105898E-2</v>
       </c>
       <c r="E8" s="1">
-        <v>2.5162613330814501E-2</v>
+        <v>2.6202247449394402E-2</v>
       </c>
       <c r="F8" s="1">
-        <v>6.3477566688662796E-3</v>
+        <v>1.32524425323044E-2</v>
       </c>
       <c r="G8" s="1">
-        <v>2.45734332225531E-3</v>
+        <v>2.74430704596349E-3</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
@@ -2512,19 +2521,19 @@
         <v>2021</v>
       </c>
       <c r="C9" s="1">
-        <v>5131</v>
+        <v>4988</v>
       </c>
       <c r="D9" s="1">
-        <v>5.7905170064019698E-2</v>
+        <v>5.96752712116378E-2</v>
       </c>
       <c r="E9" s="1">
-        <v>3.8513011257481501E-2</v>
+        <v>3.9321894512754398E-2</v>
       </c>
       <c r="F9" s="1">
-        <v>5.0596162718961604E-3</v>
+        <v>6.1146073059281597E-3</v>
       </c>
       <c r="G9" s="1">
-        <v>1.7198690047920801E-3</v>
+        <v>2.3979999820823001E-3</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
@@ -2535,19 +2544,19 @@
         <v>2022</v>
       </c>
       <c r="C10" s="1">
-        <v>5129</v>
+        <v>5025</v>
       </c>
       <c r="D10" s="1">
-        <v>4.1481101077679702E-2</v>
+        <v>4.2348282337611003E-2</v>
       </c>
       <c r="E10" s="1">
-        <v>2.7836220759408298E-2</v>
+        <v>2.34758944845175E-2</v>
       </c>
       <c r="F10" s="1">
-        <v>5.0299233281463698E-3</v>
+        <v>5.7496213197525204E-3</v>
       </c>
       <c r="G10" s="1">
-        <v>1.45964132611186E-3</v>
+        <v>1.8576312971157101E-3</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
@@ -2558,19 +2567,19 @@
         <v>2023</v>
       </c>
       <c r="C11" s="1">
-        <v>5161</v>
+        <v>5039</v>
       </c>
       <c r="D11" s="1">
-        <v>3.0554356909258999E-2</v>
+        <v>2.49298064407153E-2</v>
       </c>
       <c r="E11" s="1">
-        <v>1.65391508866429E-2</v>
+        <v>1.23782123359573E-2</v>
       </c>
       <c r="F11" s="1">
-        <v>2.5346191648455301E-3</v>
+        <v>3.36759192194673E-3</v>
       </c>
       <c r="G11" s="1">
-        <v>8.5615411174013605E-4</v>
+        <v>1.1143208973196999E-3</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
@@ -2581,16 +2590,16 @@
         <v>2024</v>
       </c>
       <c r="C12" s="1">
-        <v>5122</v>
+        <v>5011</v>
       </c>
       <c r="D12" s="1">
-        <v>2.11124203718756E-2</v>
+        <v>2.3410501443832801E-2</v>
       </c>
       <c r="E12" s="1">
-        <v>8.0262190676736404E-3</v>
+        <v>9.7182637798290394E-3</v>
       </c>
       <c r="F12" s="1">
-        <v>2.4525443207471498E-3</v>
+        <v>3.1802526645787598E-3</v>
       </c>
       <c r="G12" s="1">
         <v>0</v>
@@ -2604,16 +2613,16 @@
         <v>2025</v>
       </c>
       <c r="C13" s="1">
-        <v>5114</v>
+        <v>5001</v>
       </c>
       <c r="D13" s="1">
-        <v>1.6267060767428999E-2</v>
+        <v>1.8027354711750699E-2</v>
       </c>
       <c r="E13" s="1">
-        <v>6.3790239037187597E-3</v>
+        <v>8.2082730814930192E-3</v>
       </c>
       <c r="F13" s="1">
-        <v>2.3752838176087101E-3</v>
+        <v>3.1577195919078602E-3</v>
       </c>
       <c r="G13" s="1">
         <v>0</v>
@@ -2658,19 +2667,19 @@
         <v>2014</v>
       </c>
       <c r="C2" s="1">
-        <v>4921</v>
+        <v>4751</v>
       </c>
       <c r="D2" s="1">
-        <v>0.94480020394341302</v>
+        <v>0.95344265323662403</v>
       </c>
       <c r="E2" s="1">
-        <v>0.94732115463284905</v>
+        <v>0.97408084339902501</v>
       </c>
       <c r="F2" s="1">
-        <v>0.93901445734066302</v>
+        <v>0.93835688673275597</v>
       </c>
       <c r="G2" s="1">
-        <v>0.99766212644846497</v>
+        <v>0.99831543482838403</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
@@ -2681,19 +2690,19 @@
         <v>2015</v>
       </c>
       <c r="C3" s="1">
-        <v>5014</v>
+        <v>4848</v>
       </c>
       <c r="D3" s="1">
-        <v>0.94933445172341702</v>
+        <v>0.95161578821845905</v>
       </c>
       <c r="E3" s="1">
-        <v>0.95990762445253197</v>
+        <v>0.961985132246434</v>
       </c>
       <c r="F3" s="1">
-        <v>0.93392163392163297</v>
+        <v>0.99265229271428901</v>
       </c>
       <c r="G3" s="1">
-        <v>0.99733918712166503</v>
+        <v>0.99793601651186703</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
@@ -2704,19 +2713,19 @@
         <v>2016</v>
       </c>
       <c r="C4" s="1">
-        <v>4829</v>
+        <v>4709</v>
       </c>
       <c r="D4" s="1">
-        <v>0.93189254569785696</v>
+        <v>0.93251382424314699</v>
       </c>
       <c r="E4" s="1">
-        <v>0.90235632183907999</v>
+        <v>0.91656620990630799</v>
       </c>
       <c r="F4" s="1">
-        <v>0.98265972300841498</v>
+        <v>0.991224505592321</v>
       </c>
       <c r="G4" s="1">
-        <v>0.980984455958549</v>
+        <v>0.98905419766206104</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
@@ -2727,19 +2736,19 @@
         <v>2017</v>
       </c>
       <c r="C5" s="1">
-        <v>4946</v>
+        <v>4796</v>
       </c>
       <c r="D5" s="1">
-        <v>0.95153556821501595</v>
+        <v>0.96078502809150301</v>
       </c>
       <c r="E5" s="1">
-        <v>0.95480844080705196</v>
+        <v>0.95925652655107296</v>
       </c>
       <c r="F5" s="1">
-        <v>0.98508647480070199</v>
+        <v>0.98248501950947598</v>
       </c>
       <c r="G5" s="1">
-        <v>0.99441632928474999</v>
+        <v>0.99398051496172501</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
@@ -2750,19 +2759,19 @@
         <v>2018</v>
       </c>
       <c r="C6" s="1">
-        <v>4943</v>
+        <v>4782</v>
       </c>
       <c r="D6" s="1">
-        <v>0.95145743736773802</v>
+        <v>0.95235775801214095</v>
       </c>
       <c r="E6" s="1">
-        <v>0.95155688825642004</v>
+        <v>0.96700732100322195</v>
       </c>
       <c r="F6" s="1">
-        <v>0.98337132725430598</v>
+        <v>0.98201193967322997</v>
       </c>
       <c r="G6" s="1">
-        <v>0.994871794871794</v>
+        <v>0.99483852967845399</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
@@ -2773,19 +2782,19 @@
         <v>2019</v>
       </c>
       <c r="C7" s="1">
-        <v>4841</v>
+        <v>4699</v>
       </c>
       <c r="D7" s="1">
-        <v>0.94960985224334904</v>
+        <v>0.95842695847565496</v>
       </c>
       <c r="E7" s="1">
-        <v>0.95407780174135304</v>
+        <v>0.95175229221880198</v>
       </c>
       <c r="F7" s="1">
-        <v>0.96785861926415795</v>
+        <v>0.96021436683702399</v>
       </c>
       <c r="G7" s="1">
-        <v>0.959710743801652</v>
+        <v>0.93848446147296705</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
@@ -2796,19 +2805,19 @@
         <v>2020</v>
       </c>
       <c r="C8" s="1">
-        <v>4855</v>
+        <v>4724</v>
       </c>
       <c r="D8" s="1">
-        <v>0.95998794391688702</v>
+        <v>0.96504697637409698</v>
       </c>
       <c r="E8" s="1">
-        <v>0.95460869565217399</v>
+        <v>0.94968291125771398</v>
       </c>
       <c r="F8" s="1">
-        <v>0.98577728491850602</v>
+        <v>0.92076176844783697</v>
       </c>
       <c r="G8" s="1">
-        <v>0.997045891728496</v>
+        <v>0.99548118336510605</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
@@ -2819,19 +2828,19 @@
         <v>2021</v>
       </c>
       <c r="C9" s="1">
-        <v>5131</v>
+        <v>4988</v>
       </c>
       <c r="D9" s="1">
-        <v>0.93768816144087297</v>
+        <v>0.93489583333333304</v>
       </c>
       <c r="E9" s="1">
-        <v>0.91852079644223295</v>
+        <v>0.91416859628262104</v>
       </c>
       <c r="F9" s="1">
-        <v>0.98920310365020503</v>
+        <v>0.98226656626506004</v>
       </c>
       <c r="G9" s="1">
-        <v>0.99980499219968799</v>
+        <v>0.99872952189902997</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
@@ -2842,19 +2851,19 @@
         <v>2022</v>
       </c>
       <c r="C10" s="1">
-        <v>5129</v>
+        <v>5025</v>
       </c>
       <c r="D10" s="1">
-        <v>0.94113847622791902</v>
+        <v>0.93857687566296799</v>
       </c>
       <c r="E10" s="1">
-        <v>0.92966872563504599</v>
+        <v>0.94483764286882399</v>
       </c>
       <c r="F10" s="1">
-        <v>0.98799531524497297</v>
+        <v>0.98464169489274</v>
       </c>
       <c r="G10" s="1">
-        <v>0.99912229373902794</v>
+        <v>0.99840732629902396</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
@@ -2865,16 +2874,16 @@
         <v>2023</v>
       </c>
       <c r="C11" s="1">
-        <v>5161</v>
+        <v>5039</v>
       </c>
       <c r="D11" s="1">
-        <v>0.96021372660716897</v>
+        <v>0.97020110874569099</v>
       </c>
       <c r="E11" s="1">
-        <v>0.95243561710398394</v>
+        <v>0.97706798725860999</v>
       </c>
       <c r="F11" s="1">
-        <v>0.99932131083963505</v>
+        <v>0.99885799404170805</v>
       </c>
       <c r="G11" s="1">
         <v>1</v>
@@ -2888,16 +2897,16 @@
         <v>2024</v>
       </c>
       <c r="C12" s="1">
-        <v>5122</v>
+        <v>5011</v>
       </c>
       <c r="D12" s="1">
-        <v>0.97001374165685095</v>
+        <v>0.96510636162954</v>
       </c>
       <c r="E12" s="1">
-        <v>0.98386723822059297</v>
+        <v>0.97905454545454496</v>
       </c>
       <c r="F12" s="1">
-        <v>0.99876277918864298</v>
+        <v>0.99866879659211905</v>
       </c>
       <c r="G12" s="1"/>
     </row>
@@ -2909,16 +2918,16 @@
         <v>2025</v>
       </c>
       <c r="C13" s="1">
-        <v>5114</v>
+        <v>5001</v>
       </c>
       <c r="D13" s="1">
-        <v>0.98686955732946302</v>
+        <v>0.988670274449168</v>
       </c>
       <c r="E13" s="1">
-        <v>0.99617796942375503</v>
+        <v>0.99627513863833705</v>
       </c>
       <c r="F13" s="1">
-        <v>0.99967390595447703</v>
+        <v>0.99959983993597401</v>
       </c>
       <c r="G13" s="1"/>
     </row>
@@ -2961,19 +2970,19 @@
         <v>2014</v>
       </c>
       <c r="C2" s="1">
-        <v>4921</v>
+        <v>4751</v>
       </c>
       <c r="D2" s="1">
-        <v>0.35115021469762903</v>
+        <v>0.35894864986026798</v>
       </c>
       <c r="E2" s="1">
-        <v>0.36929093762295401</v>
+        <v>0.401971113937305</v>
       </c>
       <c r="F2" s="1">
-        <v>0.45512485144891002</v>
+        <v>0.56303860142745799</v>
       </c>
       <c r="G2" s="1">
-        <v>0.170454545454545</v>
+        <v>0.22916666666666599</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
@@ -2984,19 +2993,19 @@
         <v>2015</v>
       </c>
       <c r="C3" s="1">
-        <v>5014</v>
+        <v>4848</v>
       </c>
       <c r="D3" s="1">
-        <v>0.37069888970507697</v>
+        <v>0.39976630839314897</v>
       </c>
       <c r="E3" s="1">
-        <v>0.33366596199263698</v>
+        <v>0.34428267281978803</v>
       </c>
       <c r="F3" s="1">
-        <v>0.16626336590930799</v>
+        <v>0.28365356568167799</v>
       </c>
       <c r="G3" s="1">
-        <v>0.16254901960784299</v>
+        <v>0.27075098814229198</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
@@ -3007,19 +3016,19 @@
         <v>2016</v>
       </c>
       <c r="C4" s="1">
-        <v>4829</v>
+        <v>4709</v>
       </c>
       <c r="D4" s="1">
-        <v>0.31110876849887598</v>
+        <v>0.319557387279293</v>
       </c>
       <c r="E4" s="1">
-        <v>0.26972587264500603</v>
+        <v>0.28194045659311001</v>
       </c>
       <c r="F4" s="1">
-        <v>0.292184595865561</v>
+        <v>0.36668517981905402</v>
       </c>
       <c r="G4" s="1">
-        <v>6.4644470640920895E-2</v>
+        <v>0.168765086679833</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
@@ -3030,19 +3039,19 @@
         <v>2017</v>
       </c>
       <c r="C5" s="1">
-        <v>4946</v>
+        <v>4796</v>
       </c>
       <c r="D5" s="1">
-        <v>0.35096739615467398</v>
+        <v>0.302350380096997</v>
       </c>
       <c r="E5" s="1">
-        <v>0.33219388558840401</v>
+        <v>0.21830952737609899</v>
       </c>
       <c r="F5" s="1">
-        <v>0.19058836903742599</v>
+        <v>0.122712846769571</v>
       </c>
       <c r="G5" s="1">
-        <v>0.19704202131738299</v>
+        <v>0.12239584912832201</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
@@ -3053,19 +3062,19 @@
         <v>2018</v>
       </c>
       <c r="C6" s="1">
-        <v>4943</v>
+        <v>4782</v>
       </c>
       <c r="D6" s="1">
-        <v>0.343879574762885</v>
+        <v>0.32688112856638801</v>
       </c>
       <c r="E6" s="1">
-        <v>0.38815327449100001</v>
+        <v>0.33771751656653798</v>
       </c>
       <c r="F6" s="1">
-        <v>0.48578500676543002</v>
+        <v>0.47295544335330097</v>
       </c>
       <c r="G6" s="1">
-        <v>0.26388888888888801</v>
+        <v>0.43075117370892002</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
@@ -3076,19 +3085,19 @@
         <v>2019</v>
       </c>
       <c r="C7" s="1">
-        <v>4841</v>
+        <v>4699</v>
       </c>
       <c r="D7" s="1">
-        <v>0.32449346487441999</v>
+        <v>0.34433953826028701</v>
       </c>
       <c r="E7" s="1">
-        <v>0.28079795006231201</v>
+        <v>0.23571851700023</v>
       </c>
       <c r="F7" s="1">
-        <v>1.21271799311078E-2</v>
+        <v>1.02680482618636E-2</v>
       </c>
       <c r="G7" s="1">
-        <v>5.0761421319796898E-3</v>
+        <v>3.40136054421768E-3</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
@@ -3099,19 +3108,19 @@
         <v>2020</v>
       </c>
       <c r="C8" s="1">
-        <v>4855</v>
+        <v>4724</v>
       </c>
       <c r="D8" s="1">
-        <v>0.31021834372271101</v>
+        <v>0.31578135711674199</v>
       </c>
       <c r="E8" s="1">
-        <v>0.23654356239659999</v>
+        <v>0.26428253346214903</v>
       </c>
       <c r="F8" s="1">
-        <v>0.26458880009541902</v>
+        <v>0.395065318556514</v>
       </c>
       <c r="G8" s="1">
-        <v>0.165865384615384</v>
+        <v>0.40643274853801098</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
@@ -3122,19 +3131,19 @@
         <v>2021</v>
       </c>
       <c r="C9" s="1">
-        <v>5131</v>
+        <v>4988</v>
       </c>
       <c r="D9" s="1">
-        <v>0.39822902470691302</v>
+        <v>0.413951044708053</v>
       </c>
       <c r="E9" s="1">
-        <v>0.33086844204175297</v>
+        <v>0.38399261824358799</v>
       </c>
       <c r="F9" s="1">
-        <v>0.60428902258511197</v>
+        <v>0.58879931332040603</v>
       </c>
       <c r="G9" s="1">
-        <v>0.63888888888888795</v>
+        <v>0.24523809523809501</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
@@ -3145,19 +3154,19 @@
         <v>2022</v>
       </c>
       <c r="C10" s="1">
-        <v>5129</v>
+        <v>5025</v>
       </c>
       <c r="D10" s="1">
-        <v>0.304555560776958</v>
+        <v>0.29753686053880601</v>
       </c>
       <c r="E10" s="1">
-        <v>0.273295652667362</v>
+        <v>0.25574524945476501</v>
       </c>
       <c r="F10" s="1">
-        <v>0.283869583869583</v>
+        <v>0.24851717955047201</v>
       </c>
       <c r="G10" s="1">
-        <v>0.59090909090909005</v>
+        <v>0.308823529411764</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
@@ -3168,16 +3177,16 @@
         <v>2023</v>
       </c>
       <c r="C11" s="1">
-        <v>5161</v>
+        <v>5039</v>
       </c>
       <c r="D11" s="1">
-        <v>0.40559748005628798</v>
+        <v>0.405004518404595</v>
       </c>
       <c r="E11" s="1">
-        <v>0.37376555556616903</v>
+        <v>0.35428151838975303</v>
       </c>
       <c r="F11" s="1">
-        <v>0.54805194805194801</v>
+        <v>0.54545454545454497</v>
       </c>
       <c r="G11" s="1">
         <v>1</v>
@@ -3191,16 +3200,16 @@
         <v>2024</v>
       </c>
       <c r="C12" s="1">
-        <v>5122</v>
+        <v>5011</v>
       </c>
       <c r="D12" s="1">
-        <v>0.34167744685178603</v>
+        <v>0.33209254970896801</v>
       </c>
       <c r="E12" s="1">
-        <v>0.482392249134174</v>
+        <v>0.33882015523897402</v>
       </c>
       <c r="F12" s="1">
-        <v>0.25</v>
+        <v>0.22053872053872001</v>
       </c>
       <c r="G12" s="1">
         <v>0</v>
@@ -3214,16 +3223,16 @@
         <v>2025</v>
       </c>
       <c r="C13" s="1">
-        <v>5114</v>
+        <v>5001</v>
       </c>
       <c r="D13" s="1">
-        <v>0.61264340099625303</v>
+        <v>0.62538952244489499</v>
       </c>
       <c r="E13" s="1">
-        <v>0.755298342892046</v>
+        <v>0.74802162700483599</v>
       </c>
       <c r="F13" s="1">
-        <v>0.79166666666666596</v>
+        <v>0.68055555555555503</v>
       </c>
       <c r="G13" s="1">
         <v>0</v>
@@ -3268,19 +3277,19 @@
         <v>2014</v>
       </c>
       <c r="C2" s="1">
-        <v>4921</v>
+        <v>4751</v>
       </c>
       <c r="D2" s="1">
-        <v>0.79049894152815503</v>
+        <v>0.78613865049390197</v>
       </c>
       <c r="E2" s="1">
-        <v>0.60057846422314998</v>
+        <v>0.60425361832316105</v>
       </c>
       <c r="F2" s="1">
-        <v>0.50888931321227604</v>
+        <v>0.50922047009956795</v>
       </c>
       <c r="G2" s="1">
-        <v>0.49600149681275901</v>
+        <v>0.49712211169504</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
@@ -3291,19 +3300,19 @@
         <v>2015</v>
       </c>
       <c r="C3" s="1">
-        <v>5014</v>
+        <v>4848</v>
       </c>
       <c r="D3" s="1">
-        <v>0.81841518232205401</v>
+        <v>0.81222151838247103</v>
       </c>
       <c r="E3" s="1">
-        <v>0.56453423261997204</v>
+        <v>0.56662485578218102</v>
       </c>
       <c r="F3" s="1">
-        <v>0.50331052756414696</v>
+        <v>0.50638631167828796</v>
       </c>
       <c r="G3" s="1">
-        <v>0.49600605193270503</v>
+        <v>0.50020234059863899</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
@@ -3314,19 +3323,19 @@
         <v>2016</v>
       </c>
       <c r="C4" s="1">
-        <v>4829</v>
+        <v>4709</v>
       </c>
       <c r="D4" s="1">
-        <v>0.83158120049566397</v>
+        <v>0.80460510780238104</v>
       </c>
       <c r="E4" s="1">
-        <v>0.58307301731297001</v>
+        <v>0.57938737208004099</v>
       </c>
       <c r="F4" s="1">
-        <v>0.51119417748454199</v>
+        <v>0.51155705575874899</v>
       </c>
       <c r="G4" s="1">
-        <v>0.49280763772352798</v>
+        <v>0.48883291541593998</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
@@ -3337,19 +3346,19 @@
         <v>2017</v>
       </c>
       <c r="C5" s="1">
-        <v>4946</v>
+        <v>4796</v>
       </c>
       <c r="D5" s="1">
-        <v>0.81171748897565699</v>
+        <v>0.79901269589038104</v>
       </c>
       <c r="E5" s="1">
-        <v>0.58182078887185795</v>
+        <v>0.58017805210083495</v>
       </c>
       <c r="F5" s="1">
-        <v>0.51071964053636099</v>
+        <v>0.50227715925581495</v>
       </c>
       <c r="G5" s="1">
-        <v>0.50050768732778494</v>
+        <v>0.49800884732956102</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
@@ -3360,19 +3369,19 @@
         <v>2018</v>
       </c>
       <c r="C6" s="1">
-        <v>4943</v>
+        <v>4782</v>
       </c>
       <c r="D6" s="1">
-        <v>0.86016727534499804</v>
+        <v>0.87008853395372099</v>
       </c>
       <c r="E6" s="1">
-        <v>0.55555153521553102</v>
+        <v>0.55743370112865298</v>
       </c>
       <c r="F6" s="1">
-        <v>0.50554495696261503</v>
+        <v>0.505720078689192</v>
       </c>
       <c r="G6" s="1">
-        <v>0.50019235883871804</v>
+        <v>0.50051248219703703</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
@@ -3383,19 +3392,19 @@
         <v>2019</v>
       </c>
       <c r="C7" s="1">
-        <v>4841</v>
+        <v>4699</v>
       </c>
       <c r="D7" s="1">
-        <v>0.88820971737938204</v>
+        <v>0.90461937697363304</v>
       </c>
       <c r="E7" s="1">
-        <v>0.56637881773697296</v>
+        <v>0.56827068130608105</v>
       </c>
       <c r="F7" s="1">
-        <v>0.45460672127141</v>
+        <v>0.450032678632519</v>
       </c>
       <c r="G7" s="1">
-        <v>0.15971069115011899</v>
+        <v>0.15751378494450599</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
@@ -3406,19 +3415,19 @@
         <v>2020</v>
       </c>
       <c r="C8" s="1">
-        <v>4855</v>
+        <v>4724</v>
       </c>
       <c r="D8" s="1">
-        <v>0.81147693421240696</v>
+        <v>0.81998237638399096</v>
       </c>
       <c r="E8" s="1">
-        <v>0.56098613482114401</v>
+        <v>0.56294234531767395</v>
       </c>
       <c r="F8" s="1">
-        <v>0.50481341260208601</v>
+        <v>0.50563436126252603</v>
       </c>
       <c r="G8" s="1">
-        <v>0.49742029097373303</v>
+        <v>0.497344224071748</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
@@ -3429,19 +3438,19 @@
         <v>2021</v>
       </c>
       <c r="C9" s="1">
-        <v>5131</v>
+        <v>4988</v>
       </c>
       <c r="D9" s="1">
-        <v>0.84697517925340504</v>
+        <v>0.85736129836936104</v>
       </c>
       <c r="E9" s="1">
-        <v>0.57856852274371995</v>
+        <v>0.58092471813744695</v>
       </c>
       <c r="F9" s="1">
-        <v>0.50536469930253003</v>
+        <v>0.505506310808711</v>
       </c>
       <c r="G9" s="1">
-        <v>0.50019482709466201</v>
+        <v>0.49989762655848502</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
@@ -3452,19 +3461,19 @@
         <v>2022</v>
       </c>
       <c r="C10" s="1">
-        <v>5129</v>
+        <v>5025</v>
       </c>
       <c r="D10" s="1">
-        <v>0.667579534616911</v>
+        <v>0.67107681259101504</v>
       </c>
       <c r="E10" s="1">
-        <v>0.54439160805687103</v>
+        <v>0.54536253706087401</v>
       </c>
       <c r="F10" s="1">
-        <v>0.50279910239472903</v>
+        <v>0.50283005881430798</v>
       </c>
       <c r="G10" s="1">
-        <v>0.49830956417099198</v>
+        <v>0.49707996526002801</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
@@ -3475,19 +3484,19 @@
         <v>2023</v>
       </c>
       <c r="C11" s="1">
-        <v>5161</v>
+        <v>5039</v>
       </c>
       <c r="D11" s="1">
-        <v>0.629276097612253</v>
+        <v>0.63234664302173604</v>
       </c>
       <c r="E11" s="1">
-        <v>0.52298193803325099</v>
+        <v>0.52361966582812103</v>
       </c>
       <c r="F11" s="1">
-        <v>0.50107537927051504</v>
+        <v>0.50110040708195602</v>
       </c>
       <c r="G11" s="1">
-        <v>0.16637591166462501</v>
+        <v>0.16633579159207401</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
@@ -3498,16 +3507,16 @@
         <v>2024</v>
       </c>
       <c r="C12" s="1">
-        <v>5122</v>
+        <v>5011</v>
       </c>
       <c r="D12" s="1">
-        <v>0.57364013806553604</v>
+        <v>0.57522012835968395</v>
       </c>
       <c r="E12" s="1">
-        <v>0.51063263807566805</v>
+        <v>0.509745187287035</v>
       </c>
       <c r="F12" s="1">
-        <v>0.49960760031489199</v>
+        <v>0.49900063026879399</v>
       </c>
       <c r="G12" s="1">
         <v>0</v>
@@ -3521,16 +3530,16 @@
         <v>2025</v>
       </c>
       <c r="C13" s="1">
-        <v>5114</v>
+        <v>5001</v>
       </c>
       <c r="D13" s="1">
-        <v>0.56370258449509103</v>
+        <v>0.56516151998668096</v>
       </c>
       <c r="E13" s="1">
-        <v>0.51285093577989604</v>
+        <v>0.51314464347195998</v>
       </c>
       <c r="F13" s="1">
-        <v>0.50048897834968697</v>
+        <v>0.50049986979332195</v>
       </c>
       <c r="G13" s="1">
         <v>0</v>

</xml_diff>